<commit_message>
Generated reports are now the same, not random
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSPv2/snapshot_def_2024-02-01--2024-02-29/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSPv2/snapshot_def_2024-02-01--2024-02-29/report.xlsx
@@ -530,7 +530,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CCSP APAC Direct Reporting Template</t>
+          <t>CCSP EU Direct Reporting Template</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>info@company.org</t>
+          <t>support@partner.com</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>test_login</t>
+          <t>admin_user</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>456</t>
         </is>
       </c>
     </row>
@@ -671,28 +671,28 @@
     <row r="7" ht="25" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Customer C</t>
+          <t>Customer B</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr"/>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Lakeview</t>
+          <t>Rivertown</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>RHT1234PL</t>
+          <t>CSP8794CE</t>
         </is>
       </c>
       <c r="G7" s="8" t="n">
@@ -700,7 +700,7 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>EX: Red Hat Ansible Automation Platform, Full Support (1 Managed Node, Dedicated, Monthly)</t>
+          <t>EX: Red Hat OpenShift Container Platform, Premium Support (1 Node, Monthly)</t>
         </is>
       </c>
       <c r="I7" s="10" t="n">

</xml_diff>